<commit_message>
Add security: password, rate limit, unique projects
</commit_message>
<xml_diff>
--- a/projects/yoga-irkutsk/results/direct-import.xlsx
+++ b/projects/yoga-irkutsk/results/direct-import.xlsx
@@ -3,7 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Direct Import" sheetId="1" r:id="rId1"/>
+    <sheet name="Тексты" sheetId="1" r:id="rId1"/>
+    <sheet name="Регионы" sheetId="2" r:id="rId2"/>
+    <sheet name="Словарь значений полей" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -577,7 +579,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v/>
+        <v>Предложение текстовых блоков для кампании</v>
       </c>
       <c r="B5" t="str">
         <v/>
@@ -621,10 +623,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v/>
+        <v>Тип кампании:</v>
       </c>
       <c r="B6" t="str">
-        <v/>
+        <v>Единая перфоманс-кампания</v>
       </c>
       <c r="C6" t="str">
         <v/>
@@ -665,16 +667,16 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>№ заказа:</v>
       </c>
       <c r="B7" t="str">
         <v/>
       </c>
       <c r="C7" t="str">
-        <v/>
+        <v>Валюта:</v>
       </c>
       <c r="D7" t="str">
-        <v/>
+        <v>RUB</v>
       </c>
       <c r="E7" t="str">
         <v/>
@@ -709,7 +711,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>Минус-фразы на кампанию:</v>
       </c>
       <c r="B8" t="str">
         <v/>
@@ -836,7 +838,7 @@
         <v>0</v>
       </c>
       <c r="N10" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="11">
@@ -880,7 +882,7 @@
         <v>0</v>
       </c>
       <c r="N11" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="12">
@@ -924,7 +926,7 @@
         <v>0</v>
       </c>
       <c r="N12" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="13">
@@ -968,7 +970,7 @@
         <v>0</v>
       </c>
       <c r="N13" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="14">
@@ -1012,7 +1014,7 @@
         <v>0</v>
       </c>
       <c r="N14" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="15">
@@ -1056,7 +1058,7 @@
         <v>0</v>
       </c>
       <c r="N15" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="16">
@@ -1100,7 +1102,7 @@
         <v>0</v>
       </c>
       <c r="N16" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="17">
@@ -1144,7 +1146,7 @@
         <v>0</v>
       </c>
       <c r="N17" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="18">
@@ -1188,7 +1190,7 @@
         <v>0</v>
       </c>
       <c r="N18" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="19">
@@ -1232,7 +1234,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="20">
@@ -1276,7 +1278,7 @@
         <v>0</v>
       </c>
       <c r="N20" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="21">
@@ -1320,7 +1322,7 @@
         <v>0</v>
       </c>
       <c r="N21" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="22">
@@ -1364,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="N22" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="23">
@@ -1408,7 +1410,7 @@
         <v>0</v>
       </c>
       <c r="N23" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="24">
@@ -1452,7 +1454,7 @@
         <v>0</v>
       </c>
       <c r="N24" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="25">
@@ -1496,7 +1498,7 @@
         <v>0</v>
       </c>
       <c r="N25" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="26">
@@ -1540,7 +1542,7 @@
         <v>0</v>
       </c>
       <c r="N26" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="27">
@@ -1584,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="N27" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="28">
@@ -1628,7 +1630,7 @@
         <v>0</v>
       </c>
       <c r="N28" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="29">
@@ -1672,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="N29" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="30">
@@ -1716,7 +1718,7 @@
         <v>0</v>
       </c>
       <c r="N30" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="31">
@@ -1760,7 +1762,7 @@
         <v>0</v>
       </c>
       <c r="N31" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="32">
@@ -1804,7 +1806,7 @@
         <v>0</v>
       </c>
       <c r="N32" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="33">
@@ -1848,7 +1850,7 @@
         <v>0</v>
       </c>
       <c r="N33" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="34">
@@ -1892,7 +1894,7 @@
         <v>0</v>
       </c>
       <c r="N34" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="35">
@@ -1936,7 +1938,7 @@
         <v>0</v>
       </c>
       <c r="N35" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="36">
@@ -1980,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="N36" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
     <row r="37">
@@ -2024,7 +2026,7 @@
         <v>0</v>
       </c>
       <c r="N37" t="str">
-        <v/>
+        <v>?utm_source=yandex&amp;utm_medium=cpc&amp;utm_campaign={campaign_name}&amp;utm_term={keyword}</v>
       </c>
     </row>
   </sheetData>
@@ -2032,4 +2034,92 @@
     <ignoredError numberStoredAsText="1" sqref="A1:N37"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A3"/>
+  <sheetData>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Регионы</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Словарь значений полей</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Поле</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Допустимые значения</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Доп. объявление группы</v>
+      </c>
+      <c r="B4" t="str">
+        <v>- (основное объявление), + (дополнительное объявление)</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Тип объявления</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Текстово-графическое, Графическое, Мобильное, Видеообъявление</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Тип кампании</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Единая перфоманс-кампания, Текстово-графические объявления, Реклама приложений, Мастер кампаний</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Валюта</v>
+      </c>
+      <c r="B7" t="str">
+        <v>RUB, USD, EUR, BYN, KZT, CHF, TRY, UAH</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Длина</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Число — длина текста объявления в символах</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Комбинаторика</v>
+      </c>
+      <c r="B9" t="str">
+        <v>0 — не использовать комбинаторику, 1 — использовать</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>